<commit_message>
Initial analysis and plan for dynamic team task planner
Co-authored-by: SharksJio <124758788+SharksJio@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Team_Task_Planner.xlsx
+++ b/Team_Task_Planner.xlsx
@@ -15,7 +15,6 @@
     <sheet name="QA Team" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Weekly Planning" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="Templates" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Data Science Team" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -553,6 +552,7 @@
       </c>
     </row>
     <row r="2"/>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
@@ -561,10 +561,11 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2025-09-17 05:09</t>
-        </is>
-      </c>
-    </row>
+          <t>2025-09-17 05:48</t>
+        </is>
+      </c>
+    </row>
+    <row r="5"/>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
@@ -719,6 +720,8 @@
         <v>80</v>
       </c>
     </row>
+    <row r="11"/>
+    <row r="12"/>
     <row r="13">
       <c r="A13" s="8" t="inlineStr">
         <is>
@@ -726,6 +729,7 @@
         </is>
       </c>
     </row>
+    <row r="14"/>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
@@ -817,6 +821,7 @@
       </c>
     </row>
     <row r="2"/>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1110,6 +1115,8 @@
         </is>
       </c>
     </row>
+    <row r="11"/>
+    <row r="12"/>
     <row r="13">
       <c r="A13" s="8" t="inlineStr">
         <is>
@@ -1117,6 +1124,7 @@
         </is>
       </c>
     </row>
+    <row r="14"/>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
@@ -1189,6 +1197,7 @@
       </c>
     </row>
     <row r="2"/>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
@@ -1196,6 +1205,7 @@
         </is>
       </c>
     </row>
+    <row r="5"/>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
@@ -1430,6 +1440,8 @@
       <c r="L9" s="10" t="inlineStr"/>
       <c r="M9" s="10" t="inlineStr"/>
     </row>
+    <row r="10"/>
+    <row r="11"/>
     <row r="12">
       <c r="A12" s="8" t="inlineStr">
         <is>
@@ -1437,6 +1449,7 @@
         </is>
       </c>
     </row>
+    <row r="13"/>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
@@ -1521,6 +1534,7 @@
       </c>
     </row>
     <row r="2"/>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
@@ -1528,6 +1542,7 @@
         </is>
       </c>
     </row>
+    <row r="5"/>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
@@ -1762,6 +1777,8 @@
         </is>
       </c>
     </row>
+    <row r="10"/>
+    <row r="11"/>
     <row r="12">
       <c r="A12" s="8" t="inlineStr">
         <is>
@@ -1769,6 +1786,7 @@
         </is>
       </c>
     </row>
+    <row r="13"/>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
@@ -1853,6 +1871,7 @@
       </c>
     </row>
     <row r="2"/>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
@@ -1860,6 +1879,7 @@
         </is>
       </c>
     </row>
+    <row r="5"/>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
@@ -2094,6 +2114,8 @@
       <c r="L9" s="10" t="inlineStr"/>
       <c r="M9" s="10" t="inlineStr"/>
     </row>
+    <row r="10"/>
+    <row r="11"/>
     <row r="12">
       <c r="A12" s="8" t="inlineStr">
         <is>
@@ -2101,6 +2123,7 @@
         </is>
       </c>
     </row>
+    <row r="13"/>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
@@ -2185,6 +2208,7 @@
       </c>
     </row>
     <row r="2"/>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
@@ -2192,6 +2216,7 @@
         </is>
       </c>
     </row>
+    <row r="5"/>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
@@ -2430,6 +2455,8 @@
         </is>
       </c>
     </row>
+    <row r="10"/>
+    <row r="11"/>
     <row r="12">
       <c r="A12" s="8" t="inlineStr">
         <is>
@@ -2437,6 +2464,7 @@
         </is>
       </c>
     </row>
+    <row r="13"/>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
@@ -2516,6 +2544,7 @@
       </c>
     </row>
     <row r="2"/>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
@@ -2528,6 +2557,7 @@
         </is>
       </c>
     </row>
+    <row r="5"/>
     <row r="6">
       <c r="B6" s="3" t="inlineStr">
         <is>
@@ -2681,7 +2711,9 @@
       </c>
     </row>
     <row r="2"/>
-    <row r="4"/>
+    <row r="4">
+      <c r="A4" t="inlineStr"/>
+    </row>
     <row r="5">
       <c r="A5" s="19" t="inlineStr">
         <is>
@@ -2689,7 +2721,9 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
+    <row r="6">
+      <c r="A6" t="inlineStr"/>
+    </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
@@ -2718,7 +2752,9 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
+    <row r="11">
+      <c r="A11" t="inlineStr"/>
+    </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
@@ -2747,7 +2783,9 @@
         </is>
       </c>
     </row>
-    <row r="16"/>
+    <row r="16">
+      <c r="A16" t="inlineStr"/>
+    </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
@@ -2776,7 +2814,9 @@
         </is>
       </c>
     </row>
-    <row r="21"/>
+    <row r="21">
+      <c r="A21" t="inlineStr"/>
+    </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
@@ -2805,7 +2845,9 @@
         </is>
       </c>
     </row>
-    <row r="26"/>
+    <row r="26">
+      <c r="A26" t="inlineStr"/>
+    </row>
     <row r="27">
       <c r="A27" s="19" t="inlineStr">
         <is>
@@ -2848,7 +2890,9 @@
         </is>
       </c>
     </row>
-    <row r="33"/>
+    <row r="33">
+      <c r="A33" t="inlineStr"/>
+    </row>
     <row r="34">
       <c r="A34" s="19" t="inlineStr">
         <is>
@@ -2877,7 +2921,9 @@
         </is>
       </c>
     </row>
-    <row r="38"/>
+    <row r="38">
+      <c r="A38" t="inlineStr"/>
+    </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
@@ -2913,7 +2959,9 @@
         </is>
       </c>
     </row>
-    <row r="44"/>
+    <row r="44">
+      <c r="A44" t="inlineStr"/>
+    </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
@@ -2942,7 +2990,9 @@
         </is>
       </c>
     </row>
-    <row r="49"/>
+    <row r="49">
+      <c r="A49" t="inlineStr"/>
+    </row>
     <row r="50">
       <c r="A50" s="19" t="inlineStr">
         <is>
@@ -2991,214 +3041,4 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:M17"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="20" customWidth="1" min="12" max="12"/>
-    <col width="20" customWidth="1" min="13" max="13"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>DATA SCIENCE TEAM - TASK MANAGEMENT</t>
-        </is>
-      </c>
-    </row>
-    <row r="2"/>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>Week of: 2025-09-17</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>Task ID</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>Task Name</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>Assigned To</t>
-        </is>
-      </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>Priority</t>
-        </is>
-      </c>
-      <c r="E6" s="3" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="F6" s="3" t="inlineStr">
-        <is>
-          <t>Start Date</t>
-        </is>
-      </c>
-      <c r="G6" s="3" t="inlineStr">
-        <is>
-          <t>Due Date</t>
-        </is>
-      </c>
-      <c r="H6" s="3" t="inlineStr">
-        <is>
-          <t>Progress %</t>
-        </is>
-      </c>
-      <c r="I6" s="3" t="inlineStr">
-        <is>
-          <t>Hours Est.</t>
-        </is>
-      </c>
-      <c r="J6" s="3" t="inlineStr">
-        <is>
-          <t>Hours Actual</t>
-        </is>
-      </c>
-      <c r="K6" s="3" t="inlineStr">
-        <is>
-          <t>Dependencies</t>
-        </is>
-      </c>
-      <c r="L6" s="3" t="inlineStr">
-        <is>
-          <t>Subtasks</t>
-        </is>
-      </c>
-      <c r="M6" s="3" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="10" t="inlineStr"/>
-      <c r="B7" s="10" t="inlineStr"/>
-      <c r="C7" s="10" t="inlineStr"/>
-      <c r="D7" s="11" t="inlineStr"/>
-      <c r="E7" s="12" t="inlineStr"/>
-      <c r="F7" s="10" t="inlineStr"/>
-      <c r="G7" s="10" t="inlineStr"/>
-      <c r="H7" s="13" t="inlineStr"/>
-      <c r="I7" s="10" t="inlineStr"/>
-      <c r="J7" s="10" t="inlineStr"/>
-      <c r="K7" s="10" t="inlineStr"/>
-      <c r="L7" s="10" t="inlineStr"/>
-      <c r="M7" s="10" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="10" t="inlineStr"/>
-      <c r="B8" s="10" t="inlineStr"/>
-      <c r="C8" s="10" t="inlineStr"/>
-      <c r="D8" s="14" t="inlineStr"/>
-      <c r="E8" s="14" t="inlineStr"/>
-      <c r="F8" s="10" t="inlineStr"/>
-      <c r="G8" s="10" t="inlineStr"/>
-      <c r="H8" s="13" t="inlineStr"/>
-      <c r="I8" s="10" t="inlineStr"/>
-      <c r="J8" s="10" t="inlineStr"/>
-      <c r="K8" s="10" t="inlineStr"/>
-      <c r="L8" s="10" t="inlineStr"/>
-      <c r="M8" s="10" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="10" t="inlineStr"/>
-      <c r="B9" s="10" t="inlineStr"/>
-      <c r="C9" s="10" t="inlineStr"/>
-      <c r="D9" s="11" t="inlineStr"/>
-      <c r="E9" s="15" t="inlineStr"/>
-      <c r="F9" s="10" t="inlineStr"/>
-      <c r="G9" s="10" t="inlineStr"/>
-      <c r="H9" s="13" t="inlineStr"/>
-      <c r="I9" s="10" t="inlineStr"/>
-      <c r="J9" s="10" t="inlineStr"/>
-      <c r="K9" s="10" t="inlineStr"/>
-      <c r="L9" s="10" t="inlineStr"/>
-      <c r="M9" s="10" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="8" t="inlineStr">
-        <is>
-          <t>TEAM SUMMARY</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>Total Tasks:</t>
-        </is>
-      </c>
-      <c r="B14">
-        <f>COUNTA(A7:A9)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>Completed:</t>
-        </is>
-      </c>
-      <c r="B15">
-        <f>COUNTIF(E7:E9,"Completed")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>In Progress:</t>
-        </is>
-      </c>
-      <c r="B16" s="16">
-        <f>COUNTIF(E7:E9,"In Progress")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>Average Progress:</t>
-        </is>
-      </c>
-      <c r="B17" s="16">
-        <f>AVERAGE(H7:H9)</f>
-        <v/>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:M2"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>